<commit_message>
Fix node early stopping best model restore
</commit_message>
<xml_diff>
--- a/results/node_results.xlsx
+++ b/results/node_results.xlsx
@@ -529,13 +529,13 @@
         <v>0.7516</v>
       </c>
       <c r="L2" t="n">
-        <v>0.72</v>
+        <v>0.74</v>
       </c>
       <c r="M2" t="n">
         <v>47239</v>
       </c>
       <c r="N2" t="n">
-        <v>374.67</v>
+        <v>373.76</v>
       </c>
     </row>
     <row r="3">

</xml_diff>